<commit_message>
Update Pertanggal 8 Mei 2026 15:59 WIB
</commit_message>
<xml_diff>
--- a/Documentation/Documents/Performance Improvement/SetBulk Performance.xlsx
+++ b/Documentation/Documents/Performance Improvement/SetBulk Performance.xlsx
@@ -14,13 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
-  <si>
-    <t>TblBank</t>
-  </si>
-  <si>
-    <t>TblPerson</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
   <si>
     <t>SET</t>
   </si>
@@ -60,6 +54,42 @@
   <si>
     <t>PERFORMANCE
 INCREASE</t>
+  </si>
+  <si>
+    <t>SchMaster.TblBank</t>
+  </si>
+  <si>
+    <t>SchaMaster.TblPerson</t>
+  </si>
+  <si>
+    <t>SchSysConfig.TblAppObject_Menu</t>
+  </si>
+  <si>
+    <t>00:00:13.569</t>
+  </si>
+  <si>
+    <t>SchSysConfig.TblAppObject_MenuGroup</t>
+  </si>
+  <si>
+    <t>00:00:01.604</t>
+  </si>
+  <si>
+    <t>SchSysConfig.TblAppObject_MenuGroupMember</t>
+  </si>
+  <si>
+    <t>00:00:14.117</t>
+  </si>
+  <si>
+    <t>SchSysConfig.TblAppObject_MenuAction</t>
+  </si>
+  <si>
+    <t>00:00:08.703</t>
+  </si>
+  <si>
+    <t>SchSysConfig.TblAppObject_UserRolePrivilegesMenu</t>
+  </si>
+  <si>
+    <t>00:09:31.538</t>
   </si>
 </sst>
 </file>
@@ -466,51 +496,12 @@
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="3" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -519,9 +510,6 @@
     </xf>
     <xf numFmtId="3" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -554,6 +542,48 @@
     </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -860,11 +890,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:K11"/>
+  <dimension ref="B1:K16"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="1.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="8" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="7.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.140625" style="3" bestFit="1" customWidth="1"/>
@@ -878,191 +908,306 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="4" t="s">
+    <row r="2" spans="2:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="27" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="30" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" s="25"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="H2" s="25"/>
+      <c r="I2" s="26"/>
+      <c r="K2" s="21" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="3" spans="2:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="28"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="33" t="s">
+        <v>10</v>
+      </c>
+      <c r="E3" s="34"/>
+      <c r="F3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="33" t="s">
+        <v>10</v>
+      </c>
+      <c r="H3" s="34"/>
+      <c r="I3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K3" s="22"/>
+    </row>
+    <row r="4" spans="2:11" s="4" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="29"/>
+      <c r="C4" s="32"/>
+      <c r="D4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="E4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="K4" s="23"/>
+    </row>
+    <row r="5" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B5" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="10">
+        <v>97</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="12">
+        <f t="shared" ref="E5:E10" si="0">IF(EXACT($D5, ""), "", (RIGHT($D5, 3)*1)+(MID($D5, 7, 2)*1000)+(MID($D5, 4, 2)*1000*60)+(LEFT($D5, 2)*1000*60*60))</f>
+        <v>13569</v>
+      </c>
+      <c r="F5" s="13">
+        <f t="shared" ref="F5:F9" si="1">IF(EXACT($D5, ""), "", (E5/$C5))</f>
+        <v>139.88659793814432</v>
+      </c>
+      <c r="G5" s="11"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="13"/>
+      <c r="K5" s="14"/>
+    </row>
+    <row r="6" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B6" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="10">
+        <v>97</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="12">
+        <f t="shared" si="0"/>
+        <v>8703</v>
+      </c>
+      <c r="F6" s="13">
+        <f t="shared" si="1"/>
+        <v>89.721649484536087</v>
+      </c>
+      <c r="G6" s="11"/>
+      <c r="H6" s="12"/>
+      <c r="I6" s="13"/>
+      <c r="K6" s="14"/>
+    </row>
+    <row r="7" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B7" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="10">
+        <v>10</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="12">
+        <f t="shared" si="0"/>
+        <v>1604</v>
+      </c>
+      <c r="F7" s="13">
+        <f t="shared" si="1"/>
+        <v>160.4</v>
+      </c>
+      <c r="G7" s="11"/>
+      <c r="H7" s="12"/>
+      <c r="I7" s="13"/>
+      <c r="K7" s="14"/>
+    </row>
+    <row r="8" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B8" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="10">
+        <v>97</v>
+      </c>
+      <c r="D8" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="12">
+        <f t="shared" si="0"/>
+        <v>14117</v>
+      </c>
+      <c r="F8" s="13">
+        <f t="shared" si="1"/>
+        <v>145.53608247422682</v>
+      </c>
+      <c r="G8" s="11"/>
+      <c r="H8" s="12"/>
+      <c r="I8" s="13"/>
+      <c r="K8" s="14"/>
+    </row>
+    <row r="9" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B9" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="C9" s="10">
+        <v>2659</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="12">
+        <f t="shared" si="0"/>
+        <v>571538</v>
+      </c>
+      <c r="F9" s="13">
+        <f t="shared" si="1"/>
+        <v>214.94471605866866</v>
+      </c>
+      <c r="G9" s="11"/>
+      <c r="H9" s="12"/>
+      <c r="I9" s="13"/>
+      <c r="K9" s="14"/>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B10" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="10">
+        <v>22</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="12">
+        <f>IF(EXACT($D10, ""), "", (RIGHT($D10, 3)*1)+(MID($D10, 7, 2)*1000)+(MID($D10, 4, 2)*1000*60)+(LEFT($D10, 2)*1000*60*60))</f>
+        <v>5272</v>
+      </c>
+      <c r="F10" s="13">
+        <f>IF(EXACT($D10, ""), "", (E10/$C10))</f>
+        <v>239.63636363636363</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="H10" s="12">
+        <f>IF(EXACT($G10, ""), "", (RIGHT($G10, 3)*1)+(MID($G10, 7, 2)*1000)+(MID($G10, 4, 2)*1000*60)+(LEFT($G10, 2)*1000*60*60))</f>
+        <v>357</v>
+      </c>
+      <c r="I10" s="13">
+        <f>IF(EXACT($G10, ""), "", (H10/$C10))</f>
+        <v>16.227272727272727</v>
+      </c>
+      <c r="K10" s="14">
+        <f>IFERROR(F10/I10, "")</f>
+        <v>14.767507002801121</v>
+      </c>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B11" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="10">
+        <v>617</v>
+      </c>
+      <c r="D11" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" s="7"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="H2" s="7"/>
-      <c r="I2" s="8"/>
-      <c r="K2" s="10" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3" spans="2:11" s="9" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="11"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="14"/>
-      <c r="F3" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="G3" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="K3" s="16"/>
-    </row>
-    <row r="4" spans="2:11" s="9" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="17"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="19" t="s">
+      <c r="E11" s="12">
+        <f>IF(EXACT($D11, ""), "", (RIGHT($D11, 3)*1)+(MID($D11, 7, 2)*1000)+(MID($D11, 4, 2)*1000*60)+(LEFT($D11, 2)*1000*60*60))</f>
+        <v>156530</v>
+      </c>
+      <c r="F11" s="13">
+        <f>IF(EXACT($D11, ""), "", (E11/$C11))</f>
+        <v>253.69529983792543</v>
+      </c>
+      <c r="G11" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="E4" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="F4" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="I4" s="21" t="s">
-        <v>8</v>
-      </c>
-      <c r="K4" s="22"/>
-    </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B5" s="23" t="s">
-        <v>0</v>
-      </c>
-      <c r="C5" s="24">
-        <v>22</v>
-      </c>
-      <c r="D5" s="25" t="s">
-        <v>10</v>
-      </c>
-      <c r="E5" s="26">
-        <f>IF(EXACT($D5, ""), "", (RIGHT($D5, 3)*1)+(MID($D5, 7, 2)*1000)+(MID($D5, 4, 2)*1000*60)+(LEFT($D5, 2)*1000*60*60))</f>
-        <v>5272</v>
-      </c>
-      <c r="F5" s="27">
-        <f>IF(EXACT($D5, ""), "", (E5/$C5))</f>
-        <v>239.63636363636363</v>
-      </c>
-      <c r="G5" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="H5" s="26">
-        <f>IF(EXACT($G5, ""), "", (RIGHT($G5, 3)*1)+(MID($G5, 7, 2)*1000)+(MID($G5, 4, 2)*1000*60)+(LEFT($G5, 2)*1000*60*60))</f>
-        <v>357</v>
-      </c>
-      <c r="I5" s="27">
-        <f>IF(EXACT($G5, ""), "", (H5/$C5))</f>
-        <v>16.227272727272727</v>
-      </c>
-      <c r="K5" s="28">
-        <f>IFERROR(F5/I5, "")</f>
-        <v>14.767507002801121</v>
-      </c>
-    </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B6" s="23" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" s="24">
-        <v>617</v>
-      </c>
-      <c r="D6" s="25" t="s">
-        <v>6</v>
-      </c>
-      <c r="E6" s="26">
-        <f>IF(EXACT($D6, ""), "", (RIGHT($D6, 3)*1)+(MID($D6, 7, 2)*1000)+(MID($D6, 4, 2)*1000*60)+(LEFT($D6, 2)*1000*60*60))</f>
-        <v>156530</v>
-      </c>
-      <c r="F6" s="27">
-        <f>IF(EXACT($D6, ""), "", (E6/$C6))</f>
-        <v>253.69529983792543</v>
-      </c>
-      <c r="G6" s="25" t="s">
-        <v>9</v>
-      </c>
-      <c r="H6" s="26">
-        <f>IF(EXACT($G6, ""), "", (RIGHT($G6, 3)*1)+(MID($G6, 7, 2)*1000)+(MID($G6, 4, 2)*1000*60)+(LEFT($G6, 2)*1000*60*60))</f>
+      <c r="H11" s="12">
+        <f>IF(EXACT($G11, ""), "", (RIGHT($G11, 3)*1)+(MID($G11, 7, 2)*1000)+(MID($G11, 4, 2)*1000*60)+(LEFT($G11, 2)*1000*60*60))</f>
         <v>3322</v>
       </c>
-      <c r="I6" s="27">
-        <f>IF(EXACT($G6, ""), "", (H6/$C6))</f>
+      <c r="I11" s="13">
+        <f>IF(EXACT($G11, ""), "", (H11/$C11))</f>
         <v>5.3841166936790925</v>
       </c>
-      <c r="K6" s="28">
-        <f>IFERROR(F6/I6, "")</f>
+      <c r="K11" s="14">
+        <f>IFERROR(F11/I11, "")</f>
         <v>47.119205298013242</v>
       </c>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B7" s="23"/>
-      <c r="C7" s="24"/>
-      <c r="D7" s="25"/>
-      <c r="E7" s="26"/>
-      <c r="F7" s="29"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="26"/>
-      <c r="I7" s="29"/>
-      <c r="K7" s="24"/>
-    </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B8" s="23"/>
-      <c r="C8" s="24"/>
-      <c r="D8" s="25"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="29"/>
-      <c r="K8" s="24"/>
-    </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B9" s="23"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="25"/>
-      <c r="E9" s="26"/>
-      <c r="F9" s="29"/>
-      <c r="G9" s="25"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="29"/>
-      <c r="K9" s="24"/>
-    </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B10" s="23"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="25"/>
-      <c r="E10" s="26"/>
-      <c r="F10" s="29"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="29"/>
-      <c r="K10" s="24"/>
-    </row>
-    <row r="11" spans="2:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="30"/>
-      <c r="C11" s="31"/>
-      <c r="D11" s="32"/>
-      <c r="E11" s="33"/>
-      <c r="F11" s="34"/>
-      <c r="G11" s="32"/>
-      <c r="H11" s="33"/>
-      <c r="I11" s="34"/>
-      <c r="K11" s="31"/>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B12" s="9"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="15"/>
+      <c r="K12" s="10"/>
+    </row>
+    <row r="13" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B13" s="9"/>
+      <c r="C13" s="10"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="15"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="15"/>
+      <c r="K13" s="10"/>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B14" s="9"/>
+      <c r="C14" s="10"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="12"/>
+      <c r="I14" s="15"/>
+      <c r="K14" s="10"/>
+    </row>
+    <row r="15" spans="2:11" x14ac:dyDescent="0.2">
+      <c r="B15" s="9"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="11"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="15"/>
+      <c r="K15" s="10"/>
+    </row>
+    <row r="16" spans="2:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="16"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="18"/>
+      <c r="E16" s="19"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="19"/>
+      <c r="I16" s="20"/>
+      <c r="K16" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
Update Pertanggal 8 Juni 2026 17:01 WIB
</commit_message>
<xml_diff>
--- a/Documentation/Documents/Performance Improvement/SetBulk Performance.xlsx
+++ b/Documentation/Documents/Performance Improvement/SetBulk Performance.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="55">
   <si>
     <t>SET</t>
   </si>
@@ -120,6 +120,66 @@
   </si>
   <si>
     <t>SchMaster.TblBusinessDocumentType</t>
+  </si>
+  <si>
+    <t>SchData-OLTP-Finance.Func_TblAdvance_SET</t>
+  </si>
+  <si>
+    <t>SchMaster.TblInstitutionType</t>
+  </si>
+  <si>
+    <t>SchMaster.TblCountry</t>
+  </si>
+  <si>
+    <t>00:00:26.821</t>
+  </si>
+  <si>
+    <t>00:00:09.309</t>
+  </si>
+  <si>
+    <t>00:00:00.393</t>
+  </si>
+  <si>
+    <t>00:00:00.774</t>
+  </si>
+  <si>
+    <t>00:00:10.520</t>
+  </si>
+  <si>
+    <t>FUNCTION</t>
+  </si>
+  <si>
+    <t>SchSysConfig-Initialize.Func_SysConf_TblAppObject_Menu</t>
+  </si>
+  <si>
+    <t>SchSysConfig-Initialize.Func_SysConf_TblAppObject_MenuAction</t>
+  </si>
+  <si>
+    <t>SchSysConfig-Initialize.Func_SysConf_TblAppObject_MenuGroup</t>
+  </si>
+  <si>
+    <t>SchSysConfig-Initialize.Func_SysConf_TblAppObject_UserRolePrivilegesMenu</t>
+  </si>
+  <si>
+    <t>SchSysConfig-Initialize.Func_SysConf_TblDBObject_User</t>
+  </si>
+  <si>
+    <t>SchSysConfig-Initialize.Func_SysConf_TblAppObject_MenuMember</t>
+  </si>
+  <si>
+    <t>SchSysConfig-Initialize.Func_DtOLTP_Mstr_TblBank</t>
+  </si>
+  <si>
+    <t>SchSysConfig-Initialize.Func_DtOLTP_Mstr_TblBusinessDocumentType</t>
+  </si>
+  <si>
+    <t>SchSysConfig-Initialize.Func_DtOLTP_Mstr_TblCountry</t>
+  </si>
+  <si>
+    <t>SchSysConfig-Initialize.Func_DtOLTP_Mstr_TblInstitutionType</t>
+  </si>
+  <si>
+    <t>SchSysConfig-Initialize.Func_DtOLTP_Mstr_TblPerson</t>
   </si>
 </sst>
 </file>
@@ -155,7 +215,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -168,6 +228,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="26">
     <border>
@@ -517,7 +583,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -535,9 +601,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="3" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="3" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -548,9 +611,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -567,10 +627,25 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="47" fontId="2" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -614,6 +689,22 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -920,455 +1011,570 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:K18"/>
+  <dimension ref="B1:L19"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="1.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="38.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="2.28515625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="13.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="1"/>
+    <col min="2" max="2" width="55.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.5703125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="7.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.140625" style="18" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.140625" style="18" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="2.28515625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="13.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:11" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="2:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="27" t="s">
+    <row r="1" spans="2:12" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="2" spans="2:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B2" s="30" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="30" t="s">
+      <c r="D2" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="24" t="s">
+      <c r="E2" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="25"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="24" t="s">
+      <c r="F2" s="28"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="25"/>
-      <c r="I2" s="26"/>
-      <c r="K2" s="21" t="s">
+      <c r="I2" s="28"/>
+      <c r="J2" s="29"/>
+      <c r="L2" s="24" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="2:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="28"/>
+    <row r="3" spans="2:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="31"/>
       <c r="C3" s="31"/>
-      <c r="D3" s="33" t="s">
+      <c r="D3" s="34"/>
+      <c r="E3" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="34"/>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="37"/>
+      <c r="G3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="33" t="s">
+      <c r="H3" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="34"/>
-      <c r="I3" s="5" t="s">
+      <c r="I3" s="37"/>
+      <c r="J3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="K3" s="22"/>
-    </row>
-    <row r="4" spans="2:11" s="4" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="29"/>
+      <c r="L3" s="25"/>
+    </row>
+    <row r="4" spans="2:12" s="4" customFormat="1" ht="13.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="32"/>
       <c r="C4" s="32"/>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="35"/>
+      <c r="E4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="F4" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="G4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="H4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="I4" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="I4" s="8" t="s">
+      <c r="J4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="K4" s="23"/>
-    </row>
-    <row r="5" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B5" s="9" t="s">
+      <c r="L4" s="26"/>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B5" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="C5" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="10">
+      <c r="D5" s="9">
         <v>97</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="E5" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="12">
-        <f t="shared" ref="E5:E10" si="0">IF(EXACT($D5, ""), "", (RIGHT($D5, 3)*1)+(MID($D5, 7, 2)*1000)+(MID($D5, 4, 2)*1000*60)+(LEFT($D5, 2)*1000*60*60))</f>
+      <c r="F5" s="20">
+        <f t="shared" ref="F5:F10" si="0">IF(EXACT($E5, ""), "", (RIGHT($E5, 3)*1)+(MID($E5, 7, 2)*1000)+(MID($E5, 4, 2)*1000*60)+(LEFT($E5, 2)*1000*60*60))</f>
         <v>14586</v>
       </c>
-      <c r="F5" s="13">
-        <f t="shared" ref="F5:F9" si="1">IF(EXACT($D5, ""), "", (E5/$C5))</f>
+      <c r="G5" s="11">
+        <f t="shared" ref="G5:G9" si="1">IF(EXACT($E5, ""), "", (F5/$D5))</f>
         <v>150.37113402061857</v>
       </c>
-      <c r="G5" s="11" t="s">
+      <c r="H5" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="H5" s="12">
-        <f t="shared" ref="H5:H6" si="2">IF(EXACT($G5, ""), "", (RIGHT($G5, 3)*1)+(MID($G5, 7, 2)*1000)+(MID($G5, 4, 2)*1000*60)+(LEFT($G5, 2)*1000*60*60))</f>
+      <c r="I5" s="20">
+        <f t="shared" ref="I5:I6" si="2">IF(EXACT($H5, ""), "", (RIGHT($H5, 3)*1)+(MID($H5, 7, 2)*1000)+(MID($H5, 4, 2)*1000*60)+(LEFT($H5, 2)*1000*60*60))</f>
         <v>677</v>
       </c>
-      <c r="I5" s="13">
-        <f t="shared" ref="I5:I6" si="3">IF(EXACT($G5, ""), "", (H5/$C5))</f>
+      <c r="J5" s="11">
+        <f t="shared" ref="J5:J6" si="3">IF(EXACT($H5, ""), "", (I5/$D5))</f>
         <v>6.9793814432989691</v>
       </c>
-      <c r="K5" s="14">
-        <f t="shared" ref="K5:K6" si="4">IFERROR(F5/I5, "")</f>
+      <c r="L5" s="12">
+        <f t="shared" ref="L5:L6" si="4">IFERROR(G5/J5, "")</f>
         <v>21.545051698670608</v>
       </c>
     </row>
-    <row r="6" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B6" s="9" t="s">
+    <row r="6" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B6" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="10">
+      <c r="D6" s="9">
         <v>97</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="E6" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="12">
+      <c r="F6" s="20">
         <f t="shared" si="0"/>
         <v>15617</v>
       </c>
-      <c r="F6" s="13">
+      <c r="G6" s="11">
         <f t="shared" si="1"/>
         <v>161</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="H6" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="H6" s="12">
+      <c r="I6" s="20">
         <f t="shared" si="2"/>
         <v>767</v>
       </c>
-      <c r="I6" s="13">
+      <c r="J6" s="11">
         <f t="shared" si="3"/>
         <v>7.9072164948453612</v>
       </c>
-      <c r="K6" s="14">
+      <c r="L6" s="12">
         <f t="shared" si="4"/>
         <v>20.361147327249022</v>
       </c>
     </row>
-    <row r="7" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B7" s="9" t="s">
+    <row r="7" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B7" s="8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C7" s="10">
+      <c r="D7" s="9">
         <v>10</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="E7" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="12">
+      <c r="F7" s="20">
         <f t="shared" si="0"/>
         <v>1744</v>
       </c>
-      <c r="F7" s="13">
+      <c r="G7" s="11">
         <f t="shared" si="1"/>
         <v>174.4</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="H7" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="H7" s="12">
-        <f>IF(EXACT($G7, ""), "", (RIGHT($G7, 3)*1)+(MID($G7, 7, 2)*1000)+(MID($G7, 4, 2)*1000*60)+(LEFT($G7, 2)*1000*60*60))</f>
+      <c r="I7" s="20">
+        <f>IF(EXACT($H7, ""), "", (RIGHT($H7, 3)*1)+(MID($H7, 7, 2)*1000)+(MID($H7, 4, 2)*1000*60)+(LEFT($H7, 2)*1000*60*60))</f>
         <v>397</v>
       </c>
-      <c r="I7" s="13">
-        <f>IF(EXACT($G7, ""), "", (H7/$C7))</f>
+      <c r="J7" s="11">
+        <f>IF(EXACT($H7, ""), "", (I7/$D7))</f>
         <v>39.700000000000003</v>
       </c>
-      <c r="K7" s="14">
-        <f>IFERROR(F7/I7, "")</f>
+      <c r="L7" s="12">
+        <f>IFERROR(G7/J7, "")</f>
         <v>4.3929471032745591</v>
       </c>
     </row>
-    <row r="8" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B8" s="9" t="s">
+    <row r="8" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B8" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="10">
+      <c r="D8" s="9">
         <v>97</v>
       </c>
-      <c r="D8" s="11" t="s">
+      <c r="E8" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="12">
+      <c r="F8" s="20">
         <f t="shared" si="0"/>
         <v>15116</v>
       </c>
-      <c r="F8" s="13">
+      <c r="G8" s="11">
         <f t="shared" si="1"/>
         <v>155.83505154639175</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="H8" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="H8" s="12">
-        <f t="shared" ref="H8:H10" si="5">IF(EXACT($G8, ""), "", (RIGHT($G8, 3)*1)+(MID($G8, 7, 2)*1000)+(MID($G8, 4, 2)*1000*60)+(LEFT($G8, 2)*1000*60*60))</f>
+      <c r="I8" s="20">
+        <f t="shared" ref="I8:I10" si="5">IF(EXACT($H8, ""), "", (RIGHT($H8, 3)*1)+(MID($H8, 7, 2)*1000)+(MID($H8, 4, 2)*1000*60)+(LEFT($H8, 2)*1000*60*60))</f>
         <v>1284</v>
       </c>
-      <c r="I8" s="13">
-        <f t="shared" ref="I8:I10" si="6">IF(EXACT($G8, ""), "", (H8/$C8))</f>
+      <c r="J8" s="11">
+        <f t="shared" ref="J8:J10" si="6">IF(EXACT($H8, ""), "", (I8/$D8))</f>
         <v>13.237113402061855</v>
       </c>
-      <c r="K8" s="14">
-        <f t="shared" ref="K8:K9" si="7">IFERROR(F8/I8, "")</f>
+      <c r="L8" s="12">
+        <f t="shared" ref="L8:L9" si="7">IFERROR(G8/J8, "")</f>
         <v>11.772585669781932</v>
       </c>
     </row>
-    <row r="9" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B9" s="9" t="s">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B9" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="10">
+      <c r="D9" s="9">
         <v>2659</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="E9" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="12">
+      <c r="F9" s="20">
         <f t="shared" si="0"/>
         <v>571538</v>
       </c>
-      <c r="F9" s="13">
+      <c r="G9" s="11">
         <f t="shared" si="1"/>
         <v>214.94471605866866</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="H9" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="H9" s="12">
+      <c r="I9" s="20">
         <f t="shared" si="5"/>
         <v>14078</v>
       </c>
-      <c r="I9" s="13">
+      <c r="J9" s="11">
         <f t="shared" si="6"/>
         <v>5.2944716058668675</v>
       </c>
-      <c r="K9" s="14">
+      <c r="L9" s="12">
         <f t="shared" si="7"/>
         <v>40.597954254865741</v>
       </c>
     </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B10" s="9" t="s">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B10" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="10">
+      <c r="D10" s="9">
         <v>614</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="E10" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="E10" s="12">
+      <c r="F10" s="20">
         <f t="shared" si="0"/>
         <v>223480</v>
       </c>
-      <c r="F10" s="13">
-        <f t="shared" ref="F10" si="8">IF(EXACT($D10, ""), "", (E10/$C10))</f>
+      <c r="G10" s="11">
+        <f t="shared" ref="G10" si="8">IF(EXACT($E10, ""), "", (F10/$D10))</f>
         <v>363.97394136807816</v>
       </c>
-      <c r="G10" s="11"/>
-      <c r="H10" s="12" t="str">
+      <c r="H10" s="10"/>
+      <c r="I10" s="20" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="I10" s="13" t="str">
+      <c r="J10" s="11" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="K10" s="14" t="str">
-        <f t="shared" ref="K10" si="9">IFERROR(F10/I10, "")</f>
+      <c r="L10" s="12" t="str">
+        <f t="shared" ref="L10" si="9">IFERROR(G10/J10, "")</f>
         <v/>
       </c>
     </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B11" s="9" t="s">
+    <row r="11" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B11" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="10">
+      <c r="D11" s="9">
         <v>22</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="E11" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="E11" s="12">
-        <f>IF(EXACT($D11, ""), "", (RIGHT($D11, 3)*1)+(MID($D11, 7, 2)*1000)+(MID($D11, 4, 2)*1000*60)+(LEFT($D11, 2)*1000*60*60))</f>
+      <c r="F11" s="20">
+        <f>IF(EXACT($E11, ""), "", (RIGHT($E11, 3)*1)+(MID($E11, 7, 2)*1000)+(MID($E11, 4, 2)*1000*60)+(LEFT($E11, 2)*1000*60*60))</f>
         <v>5272</v>
       </c>
-      <c r="F11" s="13">
-        <f>IF(EXACT($D11, ""), "", (E11/$C11))</f>
+      <c r="G11" s="11">
+        <f>IF(EXACT($E11, ""), "", (F11/$D11))</f>
         <v>239.63636363636363</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="H11" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="H11" s="12">
-        <f>IF(EXACT($G11, ""), "", (RIGHT($G11, 3)*1)+(MID($G11, 7, 2)*1000)+(MID($G11, 4, 2)*1000*60)+(LEFT($G11, 2)*1000*60*60))</f>
+      <c r="I11" s="20">
+        <f>IF(EXACT($H11, ""), "", (RIGHT($H11, 3)*1)+(MID($H11, 7, 2)*1000)+(MID($H11, 4, 2)*1000*60)+(LEFT($H11, 2)*1000*60*60))</f>
         <v>357</v>
       </c>
-      <c r="I11" s="13">
-        <f>IF(EXACT($G11, ""), "", (H11/$C11))</f>
+      <c r="J11" s="11">
+        <f>IF(EXACT($H11, ""), "", (I11/$D11))</f>
         <v>16.227272727272727</v>
       </c>
-      <c r="K11" s="14">
-        <f>IFERROR(F11/I11, "")</f>
+      <c r="L11" s="12">
+        <f>IFERROR(G11/J11, "")</f>
         <v>14.767507002801121</v>
       </c>
     </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B12" s="9" t="s">
+    <row r="12" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B12" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="10">
+      <c r="D12" s="9">
         <v>148</v>
       </c>
-      <c r="D12" s="11" t="s">
+      <c r="E12" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="12">
-        <f>IF(EXACT($D12, ""), "", (RIGHT($D12, 3)*1)+(MID($D12, 7, 2)*1000)+(MID($D12, 4, 2)*1000*60)+(LEFT($D12, 2)*1000*60*60))</f>
+      <c r="F12" s="20">
+        <f>IF(EXACT($E12, ""), "", (RIGHT($E12, 3)*1)+(MID($E12, 7, 2)*1000)+(MID($E12, 4, 2)*1000*60)+(LEFT($E12, 2)*1000*60*60))</f>
         <v>32412</v>
       </c>
-      <c r="F12" s="13">
-        <f>IF(EXACT($D12, ""), "", (E12/$C12))</f>
+      <c r="G12" s="11">
+        <f>IF(EXACT($E12, ""), "", (F12/$D12))</f>
         <v>219</v>
       </c>
-      <c r="G12" s="11" t="s">
+      <c r="H12" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="H12" s="12">
-        <f>IF(EXACT($G12, ""), "", (RIGHT($G12, 3)*1)+(MID($G12, 7, 2)*1000)+(MID($G12, 4, 2)*1000*60)+(LEFT($G12, 2)*1000*60*60))</f>
+      <c r="I12" s="20">
+        <f>IF(EXACT($H12, ""), "", (RIGHT($H12, 3)*1)+(MID($H12, 7, 2)*1000)+(MID($H12, 4, 2)*1000*60)+(LEFT($H12, 2)*1000*60*60))</f>
         <v>850</v>
       </c>
-      <c r="I12" s="13">
-        <f>IF(EXACT($G12, ""), "", (H12/$C12))</f>
+      <c r="J12" s="11">
+        <f>IF(EXACT($H12, ""), "", (I12/$D12))</f>
         <v>5.743243243243243</v>
       </c>
-      <c r="K12" s="14">
-        <f>IFERROR(F12/I12, "")</f>
+      <c r="L12" s="12">
+        <f>IFERROR(G12/J12, "")</f>
         <v>38.131764705882354</v>
       </c>
     </row>
-    <row r="13" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B13" s="9" t="s">
+    <row r="13" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B13" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="9">
+        <v>197</v>
+      </c>
+      <c r="E13" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="F13" s="20">
+        <f>IF(EXACT($E13, ""), "", (RIGHT($E13, 3)*1)+(MID($E13, 7, 2)*1000)+(MID($E13, 4, 2)*1000*60)+(LEFT($E13, 2)*1000*60*60))</f>
+        <v>26821</v>
+      </c>
+      <c r="G13" s="11">
+        <f>IF(EXACT($E13, ""), "", (F13/$D13))</f>
+        <v>136.14720812182742</v>
+      </c>
+      <c r="H13" s="10"/>
+      <c r="I13" s="20"/>
+      <c r="J13" s="11"/>
+      <c r="L13" s="12"/>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B14" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="9">
+        <v>43</v>
+      </c>
+      <c r="E14" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="F14" s="20">
+        <f>IF(EXACT($E14, ""), "", (RIGHT($E14, 3)*1)+(MID($E14, 7, 2)*1000)+(MID($E14, 4, 2)*1000*60)+(LEFT($E14, 2)*1000*60*60))</f>
+        <v>9309</v>
+      </c>
+      <c r="G14" s="11">
+        <f>IF(EXACT($E14, ""), "", (F14/$D14))</f>
+        <v>216.48837209302326</v>
+      </c>
+      <c r="H14" s="22" t="s">
+        <v>40</v>
+      </c>
+      <c r="I14" s="20">
+        <f>IF(EXACT($H14, ""), "", (RIGHT($H14, 3)*1)+(MID($H14, 7, 2)*1000)+(MID($H14, 4, 2)*1000*60)+(LEFT($H14, 2)*1000*60*60))</f>
+        <v>393</v>
+      </c>
+      <c r="J14" s="11">
+        <f>IF(EXACT($H14, ""), "", (I14/$D14))</f>
+        <v>9.1395348837209305</v>
+      </c>
+      <c r="L14" s="12">
+        <f>IFERROR(G14/J14, "")</f>
+        <v>23.68702290076336</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B15" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="10">
+      <c r="D15" s="9">
         <v>617</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="E15" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E13" s="12">
-        <f>IF(EXACT($D13, ""), "", (RIGHT($D13, 3)*1)+(MID($D13, 7, 2)*1000)+(MID($D13, 4, 2)*1000*60)+(LEFT($D13, 2)*1000*60*60))</f>
+      <c r="F15" s="20">
+        <f>IF(EXACT($E15, ""), "", (RIGHT($E15, 3)*1)+(MID($E15, 7, 2)*1000)+(MID($E15, 4, 2)*1000*60)+(LEFT($E15, 2)*1000*60*60))</f>
         <v>156530</v>
       </c>
-      <c r="F13" s="13">
-        <f>IF(EXACT($D13, ""), "", (E13/$C13))</f>
+      <c r="G15" s="11">
+        <f>IF(EXACT($E15, ""), "", (F15/$D15))</f>
         <v>253.69529983792543</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="H15" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="H13" s="12">
-        <f>IF(EXACT($G13, ""), "", (RIGHT($G13, 3)*1)+(MID($G13, 7, 2)*1000)+(MID($G13, 4, 2)*1000*60)+(LEFT($G13, 2)*1000*60*60))</f>
+      <c r="I15" s="20">
+        <f>IF(EXACT($H15, ""), "", (RIGHT($H15, 3)*1)+(MID($H15, 7, 2)*1000)+(MID($H15, 4, 2)*1000*60)+(LEFT($H15, 2)*1000*60*60))</f>
         <v>3322</v>
       </c>
-      <c r="I13" s="13">
-        <f>IF(EXACT($G13, ""), "", (H13/$C13))</f>
+      <c r="J15" s="11">
+        <f>IF(EXACT($H15, ""), "", (I15/$D15))</f>
         <v>5.3841166936790925</v>
       </c>
-      <c r="K13" s="14">
-        <f>IFERROR(F13/I13, "")</f>
+      <c r="L15" s="12">
+        <f>IFERROR(G15/J15, "")</f>
         <v>47.119205298013242</v>
       </c>
     </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B14" s="9"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="11"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="15"/>
-      <c r="K14" s="10"/>
-    </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B15" s="9"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="11"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="12"/>
-      <c r="I15" s="15"/>
-      <c r="K15" s="10"/>
-    </row>
-    <row r="16" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B16" s="9"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="15"/>
-      <c r="K16" s="10"/>
-    </row>
-    <row r="17" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B17" s="9"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="12"/>
-      <c r="I17" s="15"/>
-      <c r="K17" s="10"/>
-    </row>
-    <row r="18" spans="2:11" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="16"/>
-      <c r="C18" s="17"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="19"/>
+    <row r="16" spans="2:12" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="38"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="39"/>
+      <c r="E16" s="40"/>
+      <c r="F16" s="41"/>
+      <c r="G16" s="42"/>
+      <c r="H16" s="40"/>
+      <c r="I16" s="41"/>
+      <c r="J16" s="43"/>
+      <c r="L16" s="39"/>
+    </row>
+    <row r="17" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B17" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="D17" s="9">
+        <v>1</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" s="20">
+        <f>IF(EXACT($E17, ""), "", (RIGHT($E17, 3)*1)+(MID($E17, 7, 2)*1000)+(MID($E17, 4, 2)*1000*60)+(LEFT($E17, 2)*1000*60*60))</f>
+        <v>10520</v>
+      </c>
+      <c r="G17" s="11">
+        <f>IF(EXACT($E17, ""), "", (F17/$D17))</f>
+        <v>10520</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="I17" s="20">
+        <f>IF(EXACT($H17, ""), "", (RIGHT($H17, 3)*1)+(MID($H17, 7, 2)*1000)+(MID($H17, 4, 2)*1000*60)+(LEFT($H17, 2)*1000*60*60))</f>
+        <v>774</v>
+      </c>
+      <c r="J17" s="11">
+        <f>IF(EXACT($H17, ""), "", (I17/$D17))</f>
+        <v>774</v>
+      </c>
+      <c r="L17" s="12">
+        <f>IFERROR(G17/J17, "")</f>
+        <v>13.591731266149871</v>
+      </c>
+    </row>
+    <row r="18" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="B18" s="8"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="10"/>
       <c r="F18" s="20"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="19"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="10"/>
       <c r="I18" s="20"/>
-      <c r="K18" s="17"/>
+      <c r="J18" s="13"/>
+      <c r="L18" s="9"/>
+    </row>
+    <row r="19" spans="2:12" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="16"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="16"/>
+      <c r="I19" s="21"/>
+      <c r="J19" s="17"/>
+      <c r="L19" s="15"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="K2:K4"/>
-    <mergeCell ref="D2:F2"/>
-    <mergeCell ref="G2:I2"/>
+  <mergeCells count="8">
+    <mergeCell ref="L2:L4"/>
+    <mergeCell ref="E2:G2"/>
+    <mergeCell ref="H2:J2"/>
     <mergeCell ref="B2:B4"/>
+    <mergeCell ref="D2:D4"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="H3:I3"/>
     <mergeCell ref="C2:C4"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="G3:H3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Update Pertanggal 11 Juni 2026 16:59 WIB
</commit_message>
<xml_diff>
--- a/Documentation/Documents/Performance Improvement/SetBulk Performance.xlsx
+++ b/Documentation/Documents/Performance Improvement/SetBulk Performance.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="9360" windowHeight="4620"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -215,7 +215,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -234,6 +234,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1" tint="0.34998626667073579"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="32">
     <border>
@@ -683,10 +689,6 @@
     <xf numFmtId="4" fontId="3" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -699,12 +701,57 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -738,73 +785,32 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="2" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="4" fontId="2" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -1116,13 +1122,12 @@
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="1.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="55.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.5703125" style="1" customWidth="1"/>
+    <col min="2" max="3" width="25.28515625" style="1" customWidth="1"/>
     <col min="4" max="4" width="7.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" style="15" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10" style="13" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.140625" style="11" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10" style="15" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10" style="13" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.140625" style="11" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="2.28515625" style="1" customWidth="1"/>
@@ -1133,56 +1138,56 @@
   <sheetData>
     <row r="1" spans="2:13" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:13" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="37" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="37" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="27" t="s">
+      <c r="D2" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="34" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="22"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="21" t="s">
+      <c r="F2" s="35"/>
+      <c r="G2" s="36"/>
+      <c r="H2" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="22"/>
-      <c r="J2" s="23"/>
-      <c r="L2" s="33" t="s">
+      <c r="I2" s="35"/>
+      <c r="J2" s="36"/>
+      <c r="L2" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="M2" s="34"/>
+      <c r="M2" s="29"/>
     </row>
     <row r="3" spans="2:13" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="25"/>
-      <c r="C3" s="25"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="30" t="s">
+      <c r="B3" s="38"/>
+      <c r="C3" s="38"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="31"/>
+      <c r="F3" s="44"/>
       <c r="G3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="30" t="s">
+      <c r="H3" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="31"/>
+      <c r="I3" s="44"/>
       <c r="J3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="L3" s="32"/>
-      <c r="M3" s="35"/>
+      <c r="L3" s="30"/>
+      <c r="M3" s="31"/>
     </row>
     <row r="4" spans="2:13" s="4" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="26"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="29"/>
-      <c r="E4" s="16" t="s">
+      <c r="B4" s="39"/>
+      <c r="C4" s="39"/>
+      <c r="D4" s="42"/>
+      <c r="E4" s="14" t="s">
         <v>5</v>
       </c>
       <c r="F4" s="12" t="s">
@@ -1191,7 +1196,7 @@
       <c r="G4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="H4" s="14" t="s">
         <v>5</v>
       </c>
       <c r="I4" s="12" t="s">
@@ -1200,8 +1205,8 @@
       <c r="J4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="L4" s="36"/>
-      <c r="M4" s="37"/>
+      <c r="L4" s="32"/>
+      <c r="M4" s="33"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B5" s="7" t="s">
@@ -1213,33 +1218,33 @@
       <c r="D5" s="8">
         <v>97</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="38">
+      <c r="F5" s="18">
         <f t="shared" ref="F5:F10" si="0">IF(EXACT($E5, ""), "", (RIGHT($E5, 3)*1)+(MID($E5, 7, 2)*1000)+(MID($E5, 4, 2)*1000*60)+(LEFT($E5, 2)*1000*60*60))</f>
         <v>14586</v>
       </c>
-      <c r="G5" s="39">
+      <c r="G5" s="19">
         <f t="shared" ref="G5:G9" si="1">IF(EXACT($E5, ""), "", (F5/$D5))</f>
         <v>150.37113402061857</v>
       </c>
-      <c r="H5" s="17" t="s">
+      <c r="H5" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="I5" s="38">
+      <c r="I5" s="18">
         <f t="shared" ref="I5:I6" si="2">IF(EXACT($H5, ""), "", (RIGHT($H5, 3)*1)+(MID($H5, 7, 2)*1000)+(MID($H5, 4, 2)*1000*60)+(LEFT($H5, 2)*1000*60*60))</f>
         <v>677</v>
       </c>
-      <c r="J5" s="39">
+      <c r="J5" s="19">
         <f t="shared" ref="J5:J6" si="3">IF(EXACT($H5, ""), "", (I5/$D5))</f>
         <v>6.9793814432989691</v>
       </c>
-      <c r="L5" s="46">
+      <c r="L5" s="23">
         <f t="shared" ref="L5:L6" si="4">IFERROR(G5/J5, "")</f>
         <v>21.545051698670608</v>
       </c>
-      <c r="M5" s="47" t="str">
+      <c r="M5" s="53" t="str">
         <f>IF(EXACT(L5, ""), "", CONCATENATE(TEXT(L5, "##.##"), " x"))</f>
         <v>21.55 x</v>
       </c>
@@ -1254,33 +1259,33 @@
       <c r="D6" s="8">
         <v>97</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="E6" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="38">
+      <c r="F6" s="18">
         <f t="shared" si="0"/>
         <v>15617</v>
       </c>
-      <c r="G6" s="39">
+      <c r="G6" s="19">
         <f t="shared" si="1"/>
         <v>161</v>
       </c>
-      <c r="H6" s="17" t="s">
+      <c r="H6" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="I6" s="38">
+      <c r="I6" s="18">
         <f t="shared" si="2"/>
         <v>767</v>
       </c>
-      <c r="J6" s="39">
+      <c r="J6" s="19">
         <f t="shared" si="3"/>
         <v>7.9072164948453612</v>
       </c>
-      <c r="L6" s="48">
+      <c r="L6" s="24">
         <f t="shared" si="4"/>
         <v>20.361147327249022</v>
       </c>
-      <c r="M6" s="49" t="str">
+      <c r="M6" s="25" t="str">
         <f t="shared" ref="M6:M18" si="5">IF(EXACT(L6, ""), "", CONCATENATE(TEXT(L6, "##.##"), " x"))</f>
         <v>20.36 x</v>
       </c>
@@ -1295,33 +1300,33 @@
       <c r="D7" s="8">
         <v>10</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="F7" s="38">
+      <c r="F7" s="18">
         <f t="shared" si="0"/>
         <v>1744</v>
       </c>
-      <c r="G7" s="39">
+      <c r="G7" s="19">
         <f t="shared" si="1"/>
         <v>174.4</v>
       </c>
-      <c r="H7" s="17" t="s">
+      <c r="H7" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="I7" s="38">
+      <c r="I7" s="18">
         <f>IF(EXACT($H7, ""), "", (RIGHT($H7, 3)*1)+(MID($H7, 7, 2)*1000)+(MID($H7, 4, 2)*1000*60)+(LEFT($H7, 2)*1000*60*60))</f>
         <v>397</v>
       </c>
-      <c r="J7" s="39">
+      <c r="J7" s="19">
         <f>IF(EXACT($H7, ""), "", (I7/$D7))</f>
         <v>39.700000000000003</v>
       </c>
-      <c r="L7" s="48">
+      <c r="L7" s="24">
         <f>IFERROR(G7/J7, "")</f>
         <v>4.3929471032745591</v>
       </c>
-      <c r="M7" s="49" t="str">
+      <c r="M7" s="25" t="str">
         <f t="shared" si="5"/>
         <v>4.39 x</v>
       </c>
@@ -1336,33 +1341,33 @@
       <c r="D8" s="8">
         <v>97</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="38">
+      <c r="F8" s="18">
         <f t="shared" si="0"/>
         <v>15116</v>
       </c>
-      <c r="G8" s="39">
+      <c r="G8" s="19">
         <f t="shared" si="1"/>
         <v>155.83505154639175</v>
       </c>
-      <c r="H8" s="17" t="s">
+      <c r="H8" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="I8" s="38">
+      <c r="I8" s="18">
         <f t="shared" ref="I8:I10" si="6">IF(EXACT($H8, ""), "", (RIGHT($H8, 3)*1)+(MID($H8, 7, 2)*1000)+(MID($H8, 4, 2)*1000*60)+(LEFT($H8, 2)*1000*60*60))</f>
         <v>1284</v>
       </c>
-      <c r="J8" s="39">
+      <c r="J8" s="19">
         <f t="shared" ref="J8:J10" si="7">IF(EXACT($H8, ""), "", (I8/$D8))</f>
         <v>13.237113402061855</v>
       </c>
-      <c r="L8" s="48">
+      <c r="L8" s="24">
         <f t="shared" ref="L8:L9" si="8">IFERROR(G8/J8, "")</f>
         <v>11.772585669781932</v>
       </c>
-      <c r="M8" s="49" t="str">
+      <c r="M8" s="25" t="str">
         <f t="shared" si="5"/>
         <v>11.77 x</v>
       </c>
@@ -1377,33 +1382,33 @@
       <c r="D9" s="8">
         <v>2659</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="F9" s="38">
+      <c r="F9" s="18">
         <f t="shared" si="0"/>
         <v>658431</v>
       </c>
-      <c r="G9" s="39">
+      <c r="G9" s="19">
         <f t="shared" si="1"/>
         <v>247.62354268522</v>
       </c>
-      <c r="H9" s="18" t="s">
+      <c r="H9" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="I9" s="38">
+      <c r="I9" s="18">
         <f t="shared" si="6"/>
         <v>15155</v>
       </c>
-      <c r="J9" s="39">
+      <c r="J9" s="19">
         <f t="shared" si="7"/>
         <v>5.6995110943963896</v>
       </c>
-      <c r="L9" s="48">
+      <c r="L9" s="24">
         <f t="shared" si="8"/>
         <v>43.446453315737379</v>
       </c>
-      <c r="M9" s="49" t="str">
+      <c r="M9" s="25" t="str">
         <f t="shared" si="5"/>
         <v>43.45 x</v>
       </c>
@@ -1418,31 +1423,31 @@
       <c r="D10" s="8">
         <v>614</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="38">
+      <c r="F10" s="18">
         <f t="shared" si="0"/>
         <v>223480</v>
       </c>
-      <c r="G10" s="39">
+      <c r="G10" s="19">
         <f t="shared" ref="G10" si="9">IF(EXACT($E10, ""), "", (F10/$D10))</f>
         <v>363.97394136807816</v>
       </c>
-      <c r="H10" s="17"/>
-      <c r="I10" s="38" t="str">
+      <c r="H10" s="15"/>
+      <c r="I10" s="18" t="str">
         <f t="shared" si="6"/>
         <v/>
       </c>
-      <c r="J10" s="39" t="str">
+      <c r="J10" s="19" t="str">
         <f t="shared" si="7"/>
         <v/>
       </c>
-      <c r="L10" s="48" t="str">
+      <c r="L10" s="24" t="str">
         <f t="shared" ref="L10" si="10">IFERROR(G10/J10, "")</f>
         <v/>
       </c>
-      <c r="M10" s="49" t="str">
+      <c r="M10" s="25" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -1457,33 +1462,33 @@
       <c r="D11" s="8">
         <v>22</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="38">
+      <c r="F11" s="18">
         <f>IF(EXACT($E11, ""), "", (RIGHT($E11, 3)*1)+(MID($E11, 7, 2)*1000)+(MID($E11, 4, 2)*1000*60)+(LEFT($E11, 2)*1000*60*60))</f>
         <v>5272</v>
       </c>
-      <c r="G11" s="39">
+      <c r="G11" s="19">
         <f>IF(EXACT($E11, ""), "", (F11/$D11))</f>
         <v>239.63636363636363</v>
       </c>
-      <c r="H11" s="17" t="s">
+      <c r="H11" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="I11" s="38">
+      <c r="I11" s="18">
         <f>IF(EXACT($H11, ""), "", (RIGHT($H11, 3)*1)+(MID($H11, 7, 2)*1000)+(MID($H11, 4, 2)*1000*60)+(LEFT($H11, 2)*1000*60*60))</f>
         <v>357</v>
       </c>
-      <c r="J11" s="39">
+      <c r="J11" s="19">
         <f>IF(EXACT($H11, ""), "", (I11/$D11))</f>
         <v>16.227272727272727</v>
       </c>
-      <c r="L11" s="48">
+      <c r="L11" s="24">
         <f>IFERROR(G11/J11, "")</f>
         <v>14.767507002801121</v>
       </c>
-      <c r="M11" s="49" t="str">
+      <c r="M11" s="25" t="str">
         <f t="shared" si="5"/>
         <v>14.77 x</v>
       </c>
@@ -1498,33 +1503,33 @@
       <c r="D12" s="8">
         <v>148</v>
       </c>
-      <c r="E12" s="17" t="s">
+      <c r="E12" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="F12" s="38">
+      <c r="F12" s="18">
         <f>IF(EXACT($E12, ""), "", (RIGHT($E12, 3)*1)+(MID($E12, 7, 2)*1000)+(MID($E12, 4, 2)*1000*60)+(LEFT($E12, 2)*1000*60*60))</f>
         <v>32412</v>
       </c>
-      <c r="G12" s="39">
+      <c r="G12" s="19">
         <f>IF(EXACT($E12, ""), "", (F12/$D12))</f>
         <v>219</v>
       </c>
-      <c r="H12" s="17" t="s">
+      <c r="H12" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="I12" s="38">
+      <c r="I12" s="18">
         <f>IF(EXACT($H12, ""), "", (RIGHT($H12, 3)*1)+(MID($H12, 7, 2)*1000)+(MID($H12, 4, 2)*1000*60)+(LEFT($H12, 2)*1000*60*60))</f>
         <v>850</v>
       </c>
-      <c r="J12" s="39">
+      <c r="J12" s="19">
         <f>IF(EXACT($H12, ""), "", (I12/$D12))</f>
         <v>5.743243243243243</v>
       </c>
-      <c r="L12" s="48">
+      <c r="L12" s="24">
         <f>IFERROR(G12/J12, "")</f>
         <v>38.131764705882354</v>
       </c>
-      <c r="M12" s="49" t="str">
+      <c r="M12" s="25" t="str">
         <f t="shared" si="5"/>
         <v>38.13 x</v>
       </c>
@@ -1539,22 +1544,22 @@
       <c r="D13" s="8">
         <v>197</v>
       </c>
-      <c r="E13" s="18" t="s">
+      <c r="E13" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="F13" s="38">
+      <c r="F13" s="18">
         <f>IF(EXACT($E13, ""), "", (RIGHT($E13, 3)*1)+(MID($E13, 7, 2)*1000)+(MID($E13, 4, 2)*1000*60)+(LEFT($E13, 2)*1000*60*60))</f>
         <v>26821</v>
       </c>
-      <c r="G13" s="39">
+      <c r="G13" s="19">
         <f>IF(EXACT($E13, ""), "", (F13/$D13))</f>
         <v>136.14720812182742</v>
       </c>
-      <c r="H13" s="17"/>
-      <c r="I13" s="38"/>
-      <c r="J13" s="39"/>
-      <c r="L13" s="48"/>
-      <c r="M13" s="49" t="str">
+      <c r="H13" s="15"/>
+      <c r="I13" s="18"/>
+      <c r="J13" s="19"/>
+      <c r="L13" s="24"/>
+      <c r="M13" s="25" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -1569,33 +1574,33 @@
       <c r="D14" s="8">
         <v>43</v>
       </c>
-      <c r="E14" s="18" t="s">
+      <c r="E14" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="F14" s="38">
+      <c r="F14" s="18">
         <f>IF(EXACT($E14, ""), "", (RIGHT($E14, 3)*1)+(MID($E14, 7, 2)*1000)+(MID($E14, 4, 2)*1000*60)+(LEFT($E14, 2)*1000*60*60))</f>
         <v>9309</v>
       </c>
-      <c r="G14" s="39">
+      <c r="G14" s="19">
         <f>IF(EXACT($E14, ""), "", (F14/$D14))</f>
         <v>216.48837209302326</v>
       </c>
-      <c r="H14" s="18" t="s">
+      <c r="H14" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="I14" s="38">
+      <c r="I14" s="18">
         <f>IF(EXACT($H14, ""), "", (RIGHT($H14, 3)*1)+(MID($H14, 7, 2)*1000)+(MID($H14, 4, 2)*1000*60)+(LEFT($H14, 2)*1000*60*60))</f>
         <v>393</v>
       </c>
-      <c r="J14" s="39">
+      <c r="J14" s="19">
         <f>IF(EXACT($H14, ""), "", (I14/$D14))</f>
         <v>9.1395348837209305</v>
       </c>
-      <c r="L14" s="48">
+      <c r="L14" s="24">
         <f>IFERROR(G14/J14, "")</f>
         <v>23.68702290076336</v>
       </c>
-      <c r="M14" s="49" t="str">
+      <c r="M14" s="25" t="str">
         <f t="shared" si="5"/>
         <v>23.69 x</v>
       </c>
@@ -1610,49 +1615,49 @@
       <c r="D15" s="8">
         <v>617</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="E15" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="F15" s="38">
+      <c r="F15" s="18">
         <f>IF(EXACT($E15, ""), "", (RIGHT($E15, 3)*1)+(MID($E15, 7, 2)*1000)+(MID($E15, 4, 2)*1000*60)+(LEFT($E15, 2)*1000*60*60))</f>
         <v>156530</v>
       </c>
-      <c r="G15" s="39">
+      <c r="G15" s="19">
         <f>IF(EXACT($E15, ""), "", (F15/$D15))</f>
         <v>253.69529983792543</v>
       </c>
-      <c r="H15" s="17" t="s">
+      <c r="H15" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="I15" s="38">
+      <c r="I15" s="18">
         <f>IF(EXACT($H15, ""), "", (RIGHT($H15, 3)*1)+(MID($H15, 7, 2)*1000)+(MID($H15, 4, 2)*1000*60)+(LEFT($H15, 2)*1000*60*60))</f>
         <v>3322</v>
       </c>
-      <c r="J15" s="39">
+      <c r="J15" s="19">
         <f>IF(EXACT($H15, ""), "", (I15/$D15))</f>
         <v>5.3841166936790925</v>
       </c>
-      <c r="L15" s="48">
+      <c r="L15" s="24">
         <f>IFERROR(G15/J15, "")</f>
         <v>47.119205298013242</v>
       </c>
-      <c r="M15" s="49" t="str">
+      <c r="M15" s="25" t="str">
         <f t="shared" si="5"/>
         <v>47.12 x</v>
       </c>
     </row>
-    <row r="16" spans="2:13" ht="7.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="40"/>
-      <c r="G16" s="41"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="40"/>
-      <c r="J16" s="42"/>
-      <c r="L16" s="50"/>
-      <c r="M16" s="51" t="str">
+    <row r="16" spans="2:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="45"/>
+      <c r="C16" s="45"/>
+      <c r="D16" s="46"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="48"/>
+      <c r="G16" s="49"/>
+      <c r="H16" s="47"/>
+      <c r="I16" s="48"/>
+      <c r="J16" s="50"/>
+      <c r="L16" s="51"/>
+      <c r="M16" s="52" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -1667,33 +1672,33 @@
       <c r="D17" s="8">
         <v>1</v>
       </c>
-      <c r="E17" s="17" t="s">
+      <c r="E17" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F17" s="38">
+      <c r="F17" s="18">
         <f>IF(EXACT($E17, ""), "", (RIGHT($E17, 3)*1)+(MID($E17, 7, 2)*1000)+(MID($E17, 4, 2)*1000*60)+(LEFT($E17, 2)*1000*60*60))</f>
         <v>10520</v>
       </c>
-      <c r="G17" s="39">
+      <c r="G17" s="19">
         <f>IF(EXACT($E17, ""), "", (F17/$D17))</f>
         <v>10520</v>
       </c>
-      <c r="H17" s="17" t="s">
+      <c r="H17" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="I17" s="38">
+      <c r="I17" s="18">
         <f>IF(EXACT($H17, ""), "", (RIGHT($H17, 3)*1)+(MID($H17, 7, 2)*1000)+(MID($H17, 4, 2)*1000*60)+(LEFT($H17, 2)*1000*60*60))</f>
         <v>774</v>
       </c>
-      <c r="J17" s="39">
+      <c r="J17" s="19">
         <f>IF(EXACT($H17, ""), "", (I17/$D17))</f>
         <v>774</v>
       </c>
-      <c r="L17" s="48">
+      <c r="L17" s="24">
         <f>IFERROR(G17/J17, "")</f>
         <v>13.591731266149871</v>
       </c>
-      <c r="M17" s="49" t="str">
+      <c r="M17" s="25" t="str">
         <f t="shared" si="5"/>
         <v>13.59 x</v>
       </c>
@@ -1702,14 +1707,14 @@
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
       <c r="D18" s="8"/>
-      <c r="E18" s="17"/>
-      <c r="F18" s="38"/>
-      <c r="G18" s="39"/>
-      <c r="H18" s="17"/>
-      <c r="I18" s="38"/>
-      <c r="J18" s="43"/>
-      <c r="L18" s="52"/>
-      <c r="M18" s="49" t="str">
+      <c r="E18" s="15"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="19"/>
+      <c r="H18" s="15"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="20"/>
+      <c r="L18" s="26"/>
+      <c r="M18" s="25" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
@@ -1718,17 +1723,18 @@
       <c r="B19" s="9"/>
       <c r="C19" s="9"/>
       <c r="D19" s="10"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="44"/>
-      <c r="G19" s="45"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="44"/>
-      <c r="J19" s="45"/>
-      <c r="L19" s="53"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="21"/>
+      <c r="J19" s="22"/>
+      <c r="L19" s="27"/>
       <c r="M19" s="54"/>
     </row>
   </sheetData>
   <mergeCells count="8">
+    <mergeCell ref="L2:M4"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
     <mergeCell ref="B2:B4"/>
@@ -1736,7 +1742,6 @@
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="H3:I3"/>
     <mergeCell ref="C2:C4"/>
-    <mergeCell ref="L2:M4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>

</xml_diff>

<commit_message>
Update Pertanggal 23 Juni 2026 09:36 WIB
</commit_message>
<xml_diff>
--- a/Documentation/Documents/Performance Improvement/SetBulk Performance.xlsx
+++ b/Documentation/Documents/Performance Improvement/SetBulk Performance.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="59">
   <si>
     <t>SET</t>
   </si>
@@ -180,6 +180,18 @@
   </si>
   <si>
     <t>00:00:15.155</t>
+  </si>
+  <si>
+    <t>SchSysConfig-Initialize.Func_SysConf_TblAppObject_UserRole</t>
+  </si>
+  <si>
+    <t>SchSysConfig.TblAppObject_UserRole</t>
+  </si>
+  <si>
+    <t>00:00:14.088</t>
+  </si>
+  <si>
+    <t>00:00:00.726</t>
   </si>
 </sst>
 </file>
@@ -734,57 +746,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -812,6 +773,57 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1118,11 +1130,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B1:M19"/>
+  <dimension ref="B1:M20"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="1.42578125" style="1" customWidth="1"/>
-    <col min="2" max="3" width="25.28515625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="55.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="10" style="13" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11.140625" style="11" bestFit="1" customWidth="1"/>
@@ -1138,55 +1151,55 @@
   <sheetData>
     <row r="1" spans="2:13" ht="7.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="2" spans="2:13" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="47" t="s">
         <v>41</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="40" t="s">
+      <c r="D2" s="50" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="34" t="s">
+      <c r="E2" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="35"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="34" t="s">
+      <c r="F2" s="45"/>
+      <c r="G2" s="46"/>
+      <c r="H2" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="35"/>
-      <c r="J2" s="36"/>
-      <c r="L2" s="28" t="s">
+      <c r="I2" s="45"/>
+      <c r="J2" s="46"/>
+      <c r="L2" s="38" t="s">
         <v>12</v>
       </c>
-      <c r="M2" s="29"/>
+      <c r="M2" s="39"/>
     </row>
     <row r="3" spans="2:13" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="38"/>
-      <c r="C3" s="38"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="43" t="s">
+      <c r="B3" s="48"/>
+      <c r="C3" s="48"/>
+      <c r="D3" s="51"/>
+      <c r="E3" s="53" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="44"/>
+      <c r="F3" s="54"/>
       <c r="G3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="43" t="s">
+      <c r="H3" s="53" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="44"/>
+      <c r="I3" s="54"/>
       <c r="J3" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="L3" s="30"/>
-      <c r="M3" s="31"/>
+      <c r="L3" s="40"/>
+      <c r="M3" s="41"/>
     </row>
     <row r="4" spans="2:13" s="4" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="39"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="42"/>
+      <c r="B4" s="49"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="52"/>
       <c r="E4" s="14" t="s">
         <v>5</v>
       </c>
@@ -1205,8 +1218,8 @@
       <c r="J4" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="L4" s="32"/>
-      <c r="M4" s="33"/>
+      <c r="L4" s="42"/>
+      <c r="M4" s="43"/>
     </row>
     <row r="5" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B5" s="7" t="s">
@@ -1222,11 +1235,11 @@
         <v>21</v>
       </c>
       <c r="F5" s="18">
-        <f t="shared" ref="F5:F10" si="0">IF(EXACT($E5, ""), "", (RIGHT($E5, 3)*1)+(MID($E5, 7, 2)*1000)+(MID($E5, 4, 2)*1000*60)+(LEFT($E5, 2)*1000*60*60))</f>
+        <f t="shared" ref="F5:F11" si="0">IF(EXACT($E5, ""), "", (RIGHT($E5, 3)*1)+(MID($E5, 7, 2)*1000)+(MID($E5, 4, 2)*1000*60)+(LEFT($E5, 2)*1000*60*60))</f>
         <v>14586</v>
       </c>
       <c r="G5" s="19">
-        <f t="shared" ref="G5:G9" si="1">IF(EXACT($E5, ""), "", (F5/$D5))</f>
+        <f t="shared" ref="G5:G10" si="1">IF(EXACT($E5, ""), "", (F5/$D5))</f>
         <v>150.37113402061857</v>
       </c>
       <c r="H5" s="15" t="s">
@@ -1244,8 +1257,8 @@
         <f t="shared" ref="L5:L6" si="4">IFERROR(G5/J5, "")</f>
         <v>21.545051698670608</v>
       </c>
-      <c r="M5" s="53" t="str">
-        <f>IF(EXACT(L5, ""), "", CONCATENATE(TEXT(L5, "##.##"), " x"))</f>
+      <c r="M5" s="36" t="str">
+        <f>IF(EXACT(L5, ""), "", CONCATENATE(TEXT(L5, "##.00"), " x"))</f>
         <v>21.55 x</v>
       </c>
     </row>
@@ -1286,7 +1299,7 @@
         <v>20.361147327249022</v>
       </c>
       <c r="M6" s="25" t="str">
-        <f t="shared" ref="M6:M18" si="5">IF(EXACT(L6, ""), "", CONCATENATE(TEXT(L6, "##.##"), " x"))</f>
+        <f t="shared" ref="M6:M18" si="5">IF(EXACT(L6, ""), "", CONCATENATE(TEXT(L6, "##.00"), " x"))</f>
         <v>20.36 x</v>
       </c>
     </row>
@@ -1356,15 +1369,15 @@
         <v>23</v>
       </c>
       <c r="I8" s="18">
-        <f t="shared" ref="I8:I10" si="6">IF(EXACT($H8, ""), "", (RIGHT($H8, 3)*1)+(MID($H8, 7, 2)*1000)+(MID($H8, 4, 2)*1000*60)+(LEFT($H8, 2)*1000*60*60))</f>
+        <f t="shared" ref="I8:I11" si="6">IF(EXACT($H8, ""), "", (RIGHT($H8, 3)*1)+(MID($H8, 7, 2)*1000)+(MID($H8, 4, 2)*1000*60)+(LEFT($H8, 2)*1000*60*60))</f>
         <v>1284</v>
       </c>
       <c r="J8" s="19">
-        <f t="shared" ref="J8:J10" si="7">IF(EXACT($H8, ""), "", (I8/$D8))</f>
+        <f t="shared" ref="J8:J11" si="7">IF(EXACT($H8, ""), "", (I8/$D8))</f>
         <v>13.237113402061855</v>
       </c>
       <c r="L8" s="24">
-        <f t="shared" ref="L8:L9" si="8">IFERROR(G8/J8, "")</f>
+        <f t="shared" ref="L8:L10" si="8">IFERROR(G8/J8, "")</f>
         <v>11.772585669781932</v>
       </c>
       <c r="M8" s="25" t="str">
@@ -1374,363 +1387,404 @@
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B9" s="7" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>18</v>
+        <v>56</v>
       </c>
       <c r="D9" s="8">
-        <v>2659</v>
-      </c>
-      <c r="E9" s="16" t="s">
-        <v>53</v>
+        <v>65</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>57</v>
       </c>
       <c r="F9" s="18">
         <f t="shared" si="0"/>
-        <v>658431</v>
+        <v>14088</v>
       </c>
       <c r="G9" s="19">
-        <f t="shared" si="1"/>
-        <v>247.62354268522</v>
-      </c>
-      <c r="H9" s="16" t="s">
-        <v>54</v>
+        <f t="shared" ref="G9" si="9">IF(EXACT($E9, ""), "", (F9/$D9))</f>
+        <v>216.73846153846154</v>
+      </c>
+      <c r="H9" s="15" t="s">
+        <v>58</v>
       </c>
       <c r="I9" s="18">
         <f t="shared" si="6"/>
-        <v>15155</v>
+        <v>726</v>
       </c>
       <c r="J9" s="19">
         <f t="shared" si="7"/>
-        <v>5.6995110943963896</v>
+        <v>11.169230769230769</v>
       </c>
       <c r="L9" s="24">
         <f t="shared" si="8"/>
-        <v>43.446453315737379</v>
+        <v>19.404958677685951</v>
       </c>
       <c r="M9" s="25" t="str">
         <f t="shared" si="5"/>
-        <v>43.45 x</v>
+        <v>19.40 x</v>
       </c>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B10" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="D10" s="8">
-        <v>614</v>
-      </c>
-      <c r="E10" s="15" t="s">
-        <v>28</v>
+        <v>2659</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>53</v>
       </c>
       <c r="F10" s="18">
         <f t="shared" si="0"/>
-        <v>223480</v>
+        <v>658431</v>
       </c>
       <c r="G10" s="19">
-        <f t="shared" ref="G10" si="9">IF(EXACT($E10, ""), "", (F10/$D10))</f>
-        <v>363.97394136807816</v>
-      </c>
-      <c r="H10" s="15"/>
-      <c r="I10" s="18" t="str">
+        <f t="shared" si="1"/>
+        <v>247.62354268522</v>
+      </c>
+      <c r="H10" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="I10" s="18">
         <f t="shared" si="6"/>
-        <v/>
-      </c>
-      <c r="J10" s="19" t="str">
+        <v>15155</v>
+      </c>
+      <c r="J10" s="19">
         <f t="shared" si="7"/>
-        <v/>
-      </c>
-      <c r="L10" s="24" t="str">
-        <f t="shared" ref="L10" si="10">IFERROR(G10/J10, "")</f>
-        <v/>
+        <v>5.6995110943963896</v>
+      </c>
+      <c r="L10" s="24">
+        <f t="shared" si="8"/>
+        <v>43.446453315737379</v>
       </c>
       <c r="M10" s="25" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>43.45 x</v>
       </c>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B11" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="D11" s="8">
-        <v>22</v>
+        <v>614</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="F11" s="18">
-        <f>IF(EXACT($E11, ""), "", (RIGHT($E11, 3)*1)+(MID($E11, 7, 2)*1000)+(MID($E11, 4, 2)*1000*60)+(LEFT($E11, 2)*1000*60*60))</f>
-        <v>5272</v>
+        <f t="shared" si="0"/>
+        <v>223480</v>
       </c>
       <c r="G11" s="19">
-        <f>IF(EXACT($E11, ""), "", (F11/$D11))</f>
-        <v>239.63636363636363</v>
-      </c>
-      <c r="H11" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="I11" s="18">
-        <f>IF(EXACT($H11, ""), "", (RIGHT($H11, 3)*1)+(MID($H11, 7, 2)*1000)+(MID($H11, 4, 2)*1000*60)+(LEFT($H11, 2)*1000*60*60))</f>
-        <v>357</v>
-      </c>
-      <c r="J11" s="19">
-        <f>IF(EXACT($H11, ""), "", (I11/$D11))</f>
-        <v>16.227272727272727</v>
-      </c>
-      <c r="L11" s="24">
-        <f>IFERROR(G11/J11, "")</f>
-        <v>14.767507002801121</v>
+        <f t="shared" ref="G11" si="10">IF(EXACT($E11, ""), "", (F11/$D11))</f>
+        <v>363.97394136807816</v>
+      </c>
+      <c r="H11" s="15"/>
+      <c r="I11" s="18" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="J11" s="19" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="L11" s="24" t="str">
+        <f t="shared" ref="L11" si="11">IFERROR(G11/J11, "")</f>
+        <v/>
       </c>
       <c r="M11" s="25" t="str">
         <f t="shared" si="5"/>
-        <v>14.77 x</v>
+        <v/>
       </c>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B12" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="D12" s="8">
-        <v>148</v>
+        <v>22</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F12" s="18">
         <f>IF(EXACT($E12, ""), "", (RIGHT($E12, 3)*1)+(MID($E12, 7, 2)*1000)+(MID($E12, 4, 2)*1000*60)+(LEFT($E12, 2)*1000*60*60))</f>
-        <v>32412</v>
+        <v>5272</v>
       </c>
       <c r="G12" s="19">
         <f>IF(EXACT($E12, ""), "", (F12/$D12))</f>
-        <v>219</v>
+        <v>239.63636363636363</v>
       </c>
       <c r="H12" s="15" t="s">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="I12" s="18">
         <f>IF(EXACT($H12, ""), "", (RIGHT($H12, 3)*1)+(MID($H12, 7, 2)*1000)+(MID($H12, 4, 2)*1000*60)+(LEFT($H12, 2)*1000*60*60))</f>
-        <v>850</v>
+        <v>357</v>
       </c>
       <c r="J12" s="19">
         <f>IF(EXACT($H12, ""), "", (I12/$D12))</f>
-        <v>5.743243243243243</v>
+        <v>16.227272727272727</v>
       </c>
       <c r="L12" s="24">
         <f>IFERROR(G12/J12, "")</f>
-        <v>38.131764705882354</v>
+        <v>14.767507002801121</v>
       </c>
       <c r="M12" s="25" t="str">
         <f t="shared" si="5"/>
-        <v>38.13 x</v>
+        <v>14.77 x</v>
       </c>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B13" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D13" s="8">
-        <v>197</v>
-      </c>
-      <c r="E13" s="16" t="s">
-        <v>36</v>
+        <v>148</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>30</v>
       </c>
       <c r="F13" s="18">
         <f>IF(EXACT($E13, ""), "", (RIGHT($E13, 3)*1)+(MID($E13, 7, 2)*1000)+(MID($E13, 4, 2)*1000*60)+(LEFT($E13, 2)*1000*60*60))</f>
-        <v>26821</v>
+        <v>32412</v>
       </c>
       <c r="G13" s="19">
         <f>IF(EXACT($E13, ""), "", (F13/$D13))</f>
-        <v>136.14720812182742</v>
-      </c>
-      <c r="H13" s="15"/>
-      <c r="I13" s="18"/>
-      <c r="J13" s="19"/>
-      <c r="L13" s="24"/>
+        <v>219</v>
+      </c>
+      <c r="H13" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="I13" s="18">
+        <f>IF(EXACT($H13, ""), "", (RIGHT($H13, 3)*1)+(MID($H13, 7, 2)*1000)+(MID($H13, 4, 2)*1000*60)+(LEFT($H13, 2)*1000*60*60))</f>
+        <v>850</v>
+      </c>
+      <c r="J13" s="19">
+        <f>IF(EXACT($H13, ""), "", (I13/$D13))</f>
+        <v>5.743243243243243</v>
+      </c>
+      <c r="L13" s="24">
+        <f>IFERROR(G13/J13, "")</f>
+        <v>38.131764705882354</v>
+      </c>
       <c r="M13" s="25" t="str">
         <f t="shared" si="5"/>
-        <v/>
+        <v>38.13 x</v>
       </c>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B14" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D14" s="8">
-        <v>43</v>
+        <v>197</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F14" s="18">
         <f>IF(EXACT($E14, ""), "", (RIGHT($E14, 3)*1)+(MID($E14, 7, 2)*1000)+(MID($E14, 4, 2)*1000*60)+(LEFT($E14, 2)*1000*60*60))</f>
-        <v>9309</v>
+        <v>26821</v>
       </c>
       <c r="G14" s="19">
         <f>IF(EXACT($E14, ""), "", (F14/$D14))</f>
-        <v>216.48837209302326</v>
-      </c>
-      <c r="H14" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="I14" s="18">
-        <f>IF(EXACT($H14, ""), "", (RIGHT($H14, 3)*1)+(MID($H14, 7, 2)*1000)+(MID($H14, 4, 2)*1000*60)+(LEFT($H14, 2)*1000*60*60))</f>
-        <v>393</v>
-      </c>
-      <c r="J14" s="19">
-        <f>IF(EXACT($H14, ""), "", (I14/$D14))</f>
-        <v>9.1395348837209305</v>
-      </c>
-      <c r="L14" s="24">
-        <f>IFERROR(G14/J14, "")</f>
-        <v>23.68702290076336</v>
-      </c>
+        <v>136.14720812182742</v>
+      </c>
+      <c r="H14" s="15"/>
+      <c r="I14" s="18"/>
+      <c r="J14" s="19"/>
+      <c r="L14" s="24"/>
       <c r="M14" s="25" t="str">
         <f t="shared" si="5"/>
-        <v>23.69 x</v>
+        <v/>
       </c>
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.2">
       <c r="B15" s="7" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="D15" s="8">
-        <v>617</v>
-      </c>
-      <c r="E15" s="15" t="s">
-        <v>4</v>
+        <v>43</v>
+      </c>
+      <c r="E15" s="16" t="s">
+        <v>37</v>
       </c>
       <c r="F15" s="18">
         <f>IF(EXACT($E15, ""), "", (RIGHT($E15, 3)*1)+(MID($E15, 7, 2)*1000)+(MID($E15, 4, 2)*1000*60)+(LEFT($E15, 2)*1000*60*60))</f>
-        <v>156530</v>
+        <v>9309</v>
       </c>
       <c r="G15" s="19">
         <f>IF(EXACT($E15, ""), "", (F15/$D15))</f>
-        <v>253.69529983792543</v>
-      </c>
-      <c r="H15" s="15" t="s">
-        <v>7</v>
+        <v>216.48837209302326</v>
+      </c>
+      <c r="H15" s="16" t="s">
+        <v>38</v>
       </c>
       <c r="I15" s="18">
         <f>IF(EXACT($H15, ""), "", (RIGHT($H15, 3)*1)+(MID($H15, 7, 2)*1000)+(MID($H15, 4, 2)*1000*60)+(LEFT($H15, 2)*1000*60*60))</f>
-        <v>3322</v>
+        <v>393</v>
       </c>
       <c r="J15" s="19">
         <f>IF(EXACT($H15, ""), "", (I15/$D15))</f>
-        <v>5.3841166936790925</v>
+        <v>9.1395348837209305</v>
       </c>
       <c r="L15" s="24">
         <f>IFERROR(G15/J15, "")</f>
-        <v>47.119205298013242</v>
+        <v>23.68702290076336</v>
       </c>
       <c r="M15" s="25" t="str">
         <f t="shared" si="5"/>
+        <v>23.69 x</v>
+      </c>
+    </row>
+    <row r="16" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B16" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16" s="8">
+        <v>617</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="F16" s="18">
+        <f>IF(EXACT($E16, ""), "", (RIGHT($E16, 3)*1)+(MID($E16, 7, 2)*1000)+(MID($E16, 4, 2)*1000*60)+(LEFT($E16, 2)*1000*60*60))</f>
+        <v>156530</v>
+      </c>
+      <c r="G16" s="19">
+        <f>IF(EXACT($E16, ""), "", (F16/$D16))</f>
+        <v>253.69529983792543</v>
+      </c>
+      <c r="H16" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="I16" s="18">
+        <f>IF(EXACT($H16, ""), "", (RIGHT($H16, 3)*1)+(MID($H16, 7, 2)*1000)+(MID($H16, 4, 2)*1000*60)+(LEFT($H16, 2)*1000*60*60))</f>
+        <v>3322</v>
+      </c>
+      <c r="J16" s="19">
+        <f>IF(EXACT($H16, ""), "", (I16/$D16))</f>
+        <v>5.3841166936790925</v>
+      </c>
+      <c r="L16" s="24">
+        <f>IFERROR(G16/J16, "")</f>
+        <v>47.119205298013242</v>
+      </c>
+      <c r="M16" s="25" t="str">
+        <f t="shared" si="5"/>
         <v>47.12 x</v>
       </c>
     </row>
-    <row r="16" spans="2:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="45"/>
-      <c r="C16" s="45"/>
-      <c r="D16" s="46"/>
-      <c r="E16" s="47"/>
-      <c r="F16" s="48"/>
-      <c r="G16" s="49"/>
-      <c r="H16" s="47"/>
-      <c r="I16" s="48"/>
-      <c r="J16" s="50"/>
-      <c r="L16" s="51"/>
-      <c r="M16" s="52" t="str">
+    <row r="17" spans="2:13" ht="4.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="28"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="29"/>
+      <c r="E17" s="30"/>
+      <c r="F17" s="31"/>
+      <c r="G17" s="32"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="31"/>
+      <c r="J17" s="33"/>
+      <c r="L17" s="34"/>
+      <c r="M17" s="35" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
-    <row r="17" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B17" s="7" t="s">
+    <row r="18" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B18" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="C17" s="7" t="s">
+      <c r="C18" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="D17" s="8">
+      <c r="D18" s="8">
         <v>1</v>
       </c>
-      <c r="E17" s="15" t="s">
+      <c r="E18" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="F17" s="18">
-        <f>IF(EXACT($E17, ""), "", (RIGHT($E17, 3)*1)+(MID($E17, 7, 2)*1000)+(MID($E17, 4, 2)*1000*60)+(LEFT($E17, 2)*1000*60*60))</f>
+      <c r="F18" s="18">
+        <f>IF(EXACT($E18, ""), "", (RIGHT($E18, 3)*1)+(MID($E18, 7, 2)*1000)+(MID($E18, 4, 2)*1000*60)+(LEFT($E18, 2)*1000*60*60))</f>
         <v>10520</v>
       </c>
-      <c r="G17" s="19">
-        <f>IF(EXACT($E17, ""), "", (F17/$D17))</f>
+      <c r="G18" s="19">
+        <f>IF(EXACT($E18, ""), "", (F18/$D18))</f>
         <v>10520</v>
       </c>
-      <c r="H17" s="15" t="s">
+      <c r="H18" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="I17" s="18">
-        <f>IF(EXACT($H17, ""), "", (RIGHT($H17, 3)*1)+(MID($H17, 7, 2)*1000)+(MID($H17, 4, 2)*1000*60)+(LEFT($H17, 2)*1000*60*60))</f>
+      <c r="I18" s="18">
+        <f>IF(EXACT($H18, ""), "", (RIGHT($H18, 3)*1)+(MID($H18, 7, 2)*1000)+(MID($H18, 4, 2)*1000*60)+(LEFT($H18, 2)*1000*60*60))</f>
         <v>774</v>
       </c>
-      <c r="J17" s="19">
-        <f>IF(EXACT($H17, ""), "", (I17/$D17))</f>
+      <c r="J18" s="19">
+        <f>IF(EXACT($H18, ""), "", (I18/$D18))</f>
         <v>774</v>
       </c>
-      <c r="L17" s="24">
-        <f>IFERROR(G17/J17, "")</f>
+      <c r="L18" s="24">
+        <f>IFERROR(G18/J18, "")</f>
         <v>13.591731266149871</v>
       </c>
-      <c r="M17" s="25" t="str">
+      <c r="M18" s="25" t="str">
         <f t="shared" si="5"/>
         <v>13.59 x</v>
       </c>
     </row>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.2">
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="18"/>
-      <c r="J18" s="20"/>
-      <c r="L18" s="26"/>
-      <c r="M18" s="25" t="str">
-        <f t="shared" si="5"/>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="19"/>
+      <c r="H19" s="15"/>
+      <c r="I19" s="18"/>
+      <c r="J19" s="20"/>
+      <c r="L19" s="26"/>
+      <c r="M19" s="25" t="str">
+        <f t="shared" ref="M6:M19" si="12">IF(EXACT(L19, ""), "", CONCATENATE(TEXT(L19, "##.##"), " x"))</f>
         <v/>
       </c>
     </row>
-    <row r="19" spans="2:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="21"/>
-      <c r="G19" s="22"/>
-      <c r="H19" s="17"/>
-      <c r="I19" s="21"/>
-      <c r="J19" s="22"/>
-      <c r="L19" s="27"/>
-      <c r="M19" s="54"/>
+    <row r="20" spans="2:13" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="21"/>
+      <c r="J20" s="22"/>
+      <c r="L20" s="27"/>
+      <c r="M20" s="37"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>